<commit_message>
crops simulation scripts and prelim results: crops.R
</commit_message>
<xml_diff>
--- a/Haoran/appendix_1.xlsx
+++ b/Haoran/appendix_1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="available_lands" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,9 +21,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="134">
-  <si>
-    <t xml:space="preserve">field_id</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="138">
+  <si>
+    <t xml:space="preserve">plot</t>
   </si>
   <si>
     <t xml:space="preserve">field_type</t>
@@ -377,7 +377,10 @@
     <t xml:space="preserve">crop_type</t>
   </si>
   <si>
-    <t xml:space="preserve">种植耕地</t>
+    <t xml:space="preserve">fields_growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">suitable_fields</t>
   </si>
   <si>
     <t xml:space="preserve">说明</t>
@@ -389,10 +392,7 @@
     <t xml:space="preserve">粮食（豆类）</t>
   </si>
   <si>
-    <t xml:space="preserve">平旱地
-梯田
-山坡地
-</t>
+    <t xml:space="preserve">平旱地,梯田,山坡地</t>
   </si>
   <si>
     <r>
@@ -598,6 +598,9 @@
     <t xml:space="preserve">蔬菜（豆类）</t>
   </si>
   <si>
+    <t xml:space="preserve">水浇地_1,普通大棚_1,智慧大棚_1,智慧大棚_2</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="12"/>
@@ -768,6 +771,9 @@
     <t xml:space="preserve">大白菜</t>
   </si>
   <si>
+    <t xml:space="preserve">水浇地_2</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="12"/>
@@ -810,6 +816,9 @@
   </si>
   <si>
     <t xml:space="preserve">食用菌</t>
+  </si>
+  <si>
+    <t xml:space="preserve">普通大棚_2</t>
   </si>
   <si>
     <r>
@@ -1169,7 +1178,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1249,6 +1258,12 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="宋体"/>
+      <family val="3"/>
     </font>
     <font>
       <b val="true"/>
@@ -1332,7 +1347,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1381,6 +1396,10 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1389,7 +1408,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2515,18 +2534,20 @@
     <tabColor rgb="FFF79646"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="9.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="8" width="9.36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.63"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="6" style="1" width="8.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="40.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="8" width="15.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="8" width="23.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="23.63"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="8" style="1" width="8.73"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
         <v>74</v>
       </c>
@@ -2542,595 +2563,805 @@
       <c r="E1" s="9" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F1" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="18.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E2" s="13" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="D3" s="12"/>
+        <v>81</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="E3" s="13"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="14"/>
+    </row>
+    <row r="4" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="D4" s="12"/>
+        <v>81</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="E4" s="13"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="14"/>
+    </row>
+    <row r="5" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="D5" s="12"/>
+        <v>81</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="E5" s="13"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="14"/>
+    </row>
+    <row r="6" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="D6" s="12"/>
+        <v>81</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="E6" s="13"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="14"/>
+    </row>
+    <row r="7" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D7" s="12"/>
+        <v>89</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="E7" s="13"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="14"/>
+    </row>
+    <row r="8" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D8" s="12"/>
+      <c r="D8" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="E8" s="13"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="14"/>
+    </row>
+    <row r="9" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D9" s="12"/>
+        <v>89</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="E9" s="13"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="14"/>
+    </row>
+    <row r="10" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D10" s="12"/>
+        <v>89</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="E10" s="13"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="14"/>
+    </row>
+    <row r="11" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D11" s="12"/>
+        <v>89</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="E11" s="13"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="14"/>
+    </row>
+    <row r="12" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D12" s="12"/>
+        <v>89</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="E12" s="13"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="14"/>
+    </row>
+    <row r="13" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D13" s="12"/>
+        <v>89</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="E13" s="13"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="14"/>
+    </row>
+    <row r="14" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D14" s="12"/>
+        <v>89</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="E14" s="13"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="14"/>
+    </row>
+    <row r="15" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D15" s="12"/>
+        <v>89</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="E15" s="13"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="14"/>
+    </row>
+    <row r="16" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="n">
         <v>15</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D16" s="12"/>
+        <v>89</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="E16" s="13"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="14"/>
+    </row>
+    <row r="17" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="n">
         <v>16</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D17" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D17" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="E17" s="13"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E17" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="14"/>
+    </row>
+    <row r="18" customFormat="false" ht="18.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="n">
         <v>17</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="E18" s="13"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>102</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="F18" s="6"/>
+      <c r="G18" s="14"/>
+    </row>
+    <row r="19" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="n">
         <v>18</v>
       </c>
       <c r="B19" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="D19" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="C19" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="D19" s="12"/>
       <c r="E19" s="13"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F19" s="3"/>
+      <c r="G19" s="14"/>
+    </row>
+    <row r="20" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="n">
         <v>19</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="D20" s="12"/>
+        <v>101</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E20" s="13"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F20" s="3"/>
+      <c r="G20" s="14"/>
+    </row>
+    <row r="21" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="n">
         <v>20</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D21" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E21" s="13"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F21" s="3"/>
+      <c r="G21" s="14"/>
+    </row>
+    <row r="22" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="n">
         <v>21</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D22" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E22" s="13"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F22" s="3"/>
+      <c r="G22" s="14"/>
+    </row>
+    <row r="23" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="n">
         <v>22</v>
       </c>
       <c r="B23" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="C23" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="C23" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D23" s="12"/>
+      <c r="D23" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E23" s="13"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F23" s="3"/>
+      <c r="G23" s="14"/>
+    </row>
+    <row r="24" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="n">
         <v>23</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D24" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E24" s="13"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F24" s="3"/>
+      <c r="G24" s="14"/>
+    </row>
+    <row r="25" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="n">
         <v>24</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D25" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E25" s="13"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F25" s="3"/>
+      <c r="G25" s="14"/>
+    </row>
+    <row r="26" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="n">
         <v>25</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D26" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E26" s="13"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F26" s="3"/>
+      <c r="G26" s="14"/>
+    </row>
+    <row r="27" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="n">
         <v>26</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D27" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E27" s="13"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F27" s="3"/>
+      <c r="G27" s="14"/>
+    </row>
+    <row r="28" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="n">
         <v>27</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D28" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E28" s="13"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F28" s="3"/>
+      <c r="G28" s="14"/>
+    </row>
+    <row r="29" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="n">
         <v>28</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D29" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E29" s="13"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F29" s="3"/>
+      <c r="G29" s="14"/>
+    </row>
+    <row r="30" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="n">
         <v>29</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D30" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E30" s="13"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F30" s="3"/>
+      <c r="G30" s="14"/>
+    </row>
+    <row r="31" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="n">
         <v>30</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D31" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E31" s="13"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F31" s="3"/>
+      <c r="G31" s="14"/>
+    </row>
+    <row r="32" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="n">
         <v>31</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D32" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E32" s="13"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F32" s="3"/>
+      <c r="G32" s="14"/>
+    </row>
+    <row r="33" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="n">
         <v>32</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D33" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E33" s="13"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F33" s="3"/>
+      <c r="G33" s="14"/>
+    </row>
+    <row r="34" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="n">
         <v>33</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D34" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E34" s="13"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F34" s="3"/>
+      <c r="G34" s="14"/>
+    </row>
+    <row r="35" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="n">
         <v>34</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D35" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="E35" s="13"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="14"/>
     </row>
     <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="n">
         <v>35</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="E36" s="13"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>123</v>
+      </c>
+      <c r="E36" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="F36" s="6"/>
+      <c r="G36" s="14"/>
+    </row>
+    <row r="37" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="n">
         <v>36</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D37" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>123</v>
+      </c>
       <c r="E37" s="13"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F37" s="6"/>
+      <c r="G37" s="14"/>
+    </row>
+    <row r="38" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="n">
         <v>37</v>
       </c>
       <c r="B38" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C38" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="D38" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="C38" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D38" s="12"/>
       <c r="E38" s="13"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F38" s="6"/>
+      <c r="G38" s="14"/>
+    </row>
+    <row r="39" customFormat="false" ht="18.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="n">
         <v>38</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="E39" s="13"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>129</v>
+      </c>
+      <c r="E39" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="F39" s="6"/>
+      <c r="G39" s="14"/>
+    </row>
+    <row r="40" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="n">
         <v>39</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="D40" s="12"/>
+        <v>128</v>
+      </c>
+      <c r="D40" s="12" t="s">
+        <v>129</v>
+      </c>
       <c r="E40" s="13"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F40" s="6"/>
+      <c r="G40" s="14"/>
+    </row>
+    <row r="41" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="n">
         <v>40</v>
       </c>
       <c r="B41" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="C41" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="C41" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="D41" s="12"/>
+      <c r="D41" s="12" t="s">
+        <v>129</v>
+      </c>
       <c r="E41" s="13"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F41" s="6"/>
+      <c r="G41" s="14"/>
+    </row>
+    <row r="42" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="n">
         <v>41</v>
       </c>
       <c r="B42" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="C42" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="D42" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="C42" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="D42" s="12"/>
       <c r="E42" s="13"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="14"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="14"/>
-      <c r="B43" s="15"/>
-      <c r="C43" s="15"/>
+      <c r="A43" s="15"/>
+      <c r="B43" s="16"/>
+      <c r="C43" s="16"/>
       <c r="D43" s="16"/>
-      <c r="E43" s="15"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="17" t="s">
-        <v>130</v>
-      </c>
-      <c r="B44" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="C44" s="15"/>
+      <c r="E43" s="17"/>
+      <c r="F43" s="17"/>
+      <c r="G43" s="16"/>
+    </row>
+    <row r="44" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="B44" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="C44" s="16"/>
       <c r="D44" s="16"/>
-      <c r="E44" s="15"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="14"/>
-      <c r="B45" s="18" t="s">
-        <v>132</v>
-      </c>
-      <c r="C45" s="15"/>
+      <c r="E44" s="17"/>
+      <c r="F44" s="17"/>
+      <c r="G44" s="16"/>
+    </row>
+    <row r="45" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="15"/>
+      <c r="B45" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="C45" s="16"/>
       <c r="D45" s="16"/>
-      <c r="E45" s="15"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="14"/>
-      <c r="B46" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="C46" s="15"/>
+      <c r="E45" s="17"/>
+      <c r="F45" s="17"/>
+      <c r="G45" s="16"/>
+    </row>
+    <row r="46" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="15"/>
+      <c r="B46" s="19" t="s">
+        <v>137</v>
+      </c>
+      <c r="C46" s="16"/>
       <c r="D46" s="16"/>
-      <c r="E46" s="15"/>
+      <c r="E46" s="17"/>
+      <c r="F46" s="17"/>
+      <c r="G46" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="D2:D16"/>
-    <mergeCell ref="E2:E42"/>
-    <mergeCell ref="D18:D35"/>
-    <mergeCell ref="D36:D38"/>
-    <mergeCell ref="D39:D42"/>
+    <mergeCell ref="E2:E16"/>
+    <mergeCell ref="G2:G42"/>
+    <mergeCell ref="E18:E35"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="E39:E42"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>